<commit_message>
Descripción de lo que has cambiado
</commit_message>
<xml_diff>
--- a/AULAS/IF04/if04-NOMBRE-IP-MAC.xlsx
+++ b/AULAS/IF04/if04-NOMBRE-IP-MAC.xlsx
@@ -1,11 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="30219"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="30026"/>
   <workbookPr defaultThemeVersion="166925"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{01C9F579-64B7-4A21-AB99-B875133CAE80}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\angelica\GITHUB\informatica-iesmhp\AULAS2627\AULAS\IF04\"/>
+    </mc:Choice>
+  </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4B894F79-AC12-4F49-BF8C-815D5E160127}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="240" yWindow="105" windowWidth="14805" windowHeight="8010" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="19090" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Hoja1" sheetId="1" r:id="rId1"/>
@@ -31,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="117" uniqueCount="68">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="159" uniqueCount="74">
   <si>
     <t>Estado</t>
   </si>
@@ -69,9 +74,6 @@
     <t>30:9C:23:40:39:C7</t>
   </si>
   <si>
-    <t>Micro-Star INTL CO., LTD.</t>
-  </si>
-  <si>
     <t>IF04-01</t>
   </si>
   <si>
@@ -235,16 +237,43 @@
   </si>
   <si>
     <t>7C:10:C9:84:CC:26</t>
+  </si>
+  <si>
+    <t>IF04-17</t>
+  </si>
+  <si>
+    <t>MSI-H110 M-PRO-VH</t>
+  </si>
+  <si>
+    <t>16GB</t>
+  </si>
+  <si>
+    <t>SSD SATA 1TB</t>
+  </si>
+  <si>
+    <t xml:space="preserve">SATA 1TB </t>
+  </si>
+  <si>
+    <t>ASUS PRIME H510-R R2.0</t>
+  </si>
+  <si>
+    <t>7C:10:C9:84:C3:75</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="1">
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="8"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -290,9 +319,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office 2013 - Tema de 2022">
   <a:themeElements>
-    <a:clrScheme name="Office">
+    <a:clrScheme name="Office 2013 - 2022">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -330,7 +359,7 @@
         <a:srgbClr val="954F72"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office">
+    <a:fontScheme name="Office 2013 - 2022">
       <a:majorFont>
         <a:latin typeface="Calibri Light" panose="020F0302020204030204"/>
         <a:ea typeface=""/>
@@ -436,7 +465,7 @@
         <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office">
+    <a:fmtScheme name="Office 2013 - 2022">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -578,7 +607,7 @@
   <a:extraClrSchemeLst/>
   <a:extLst>
     <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
+      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office 2013 - 2022 Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
     </a:ext>
   </a:extLst>
 </a:theme>
@@ -586,19 +615,19 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:H19"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <dimension ref="A1:H20"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="9.23046875" defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
   <cols>
-    <col min="2" max="2" width="8.85546875" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="10.42578125" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="23.85546875" customWidth="1"/>
-    <col min="5" max="5" width="20.85546875" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="14.42578125" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="13.28515625" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="24.42578125" customWidth="1"/>
+    <col min="2" max="2" width="8.84375" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="10.3828125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="16.15234375" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="21.53515625" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="14.3828125" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="13.3046875" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="24.3828125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8">
+    <row r="1" spans="1:8" x14ac:dyDescent="0.4">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -624,7 +653,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="2" spans="1:8">
+    <row r="2" spans="1:8" x14ac:dyDescent="0.4">
       <c r="A2" t="s">
         <v>8</v>
       </c>
@@ -638,356 +667,485 @@
         <v>11</v>
       </c>
       <c r="E2" t="s">
+        <v>68</v>
+      </c>
+      <c r="F2" t="s">
+        <v>69</v>
+      </c>
+      <c r="G2" t="s">
+        <v>70</v>
+      </c>
+      <c r="H2" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="3" spans="1:8" x14ac:dyDescent="0.4">
+      <c r="A3" t="s">
+        <v>8</v>
+      </c>
+      <c r="B3" t="s">
         <v>12</v>
       </c>
-    </row>
-    <row r="3" spans="1:8">
-      <c r="A3" t="s">
-        <v>8</v>
-      </c>
-      <c r="B3" t="s">
+      <c r="C3" t="s">
         <v>13</v>
       </c>
-      <c r="C3" t="s">
+      <c r="D3" t="s">
         <v>14</v>
       </c>
-      <c r="D3" t="s">
+      <c r="E3" t="s">
+        <v>39</v>
+      </c>
+      <c r="F3" t="s">
+        <v>40</v>
+      </c>
+      <c r="G3" t="s">
+        <v>41</v>
+      </c>
+      <c r="H3" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="4" spans="1:8" x14ac:dyDescent="0.4">
+      <c r="A4" t="s">
+        <v>8</v>
+      </c>
+      <c r="B4" t="s">
         <v>15</v>
       </c>
-    </row>
-    <row r="4" spans="1:8">
-      <c r="A4" t="s">
-        <v>8</v>
-      </c>
-      <c r="B4" t="s">
+      <c r="C4" t="s">
         <v>16</v>
       </c>
-      <c r="C4" t="s">
+      <c r="D4" t="s">
         <v>17</v>
       </c>
-      <c r="D4" t="s">
+      <c r="E4" t="s">
+        <v>39</v>
+      </c>
+      <c r="F4" t="s">
+        <v>40</v>
+      </c>
+      <c r="G4" t="s">
+        <v>41</v>
+      </c>
+      <c r="H4" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="5" spans="1:8" x14ac:dyDescent="0.4">
+      <c r="A5" t="s">
+        <v>8</v>
+      </c>
+      <c r="B5" t="s">
         <v>18</v>
       </c>
-    </row>
-    <row r="5" spans="1:8">
-      <c r="A5" t="s">
-        <v>8</v>
-      </c>
-      <c r="B5" t="s">
+      <c r="C5" t="s">
         <v>19</v>
       </c>
-      <c r="C5" t="s">
+      <c r="D5" t="s">
         <v>20</v>
       </c>
-      <c r="D5" t="s">
+      <c r="E5" t="s">
+        <v>39</v>
+      </c>
+      <c r="F5" t="s">
+        <v>40</v>
+      </c>
+      <c r="G5" t="s">
+        <v>41</v>
+      </c>
+      <c r="H5" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="6" spans="1:8" x14ac:dyDescent="0.4">
+      <c r="A6" t="s">
+        <v>8</v>
+      </c>
+      <c r="B6" t="s">
         <v>21</v>
       </c>
-    </row>
-    <row r="6" spans="1:8">
-      <c r="A6" t="s">
-        <v>8</v>
-      </c>
-      <c r="B6" t="s">
+      <c r="C6" t="s">
         <v>22</v>
       </c>
-      <c r="C6" t="s">
+      <c r="D6" t="s">
         <v>23</v>
       </c>
-      <c r="D6" t="s">
+      <c r="E6" t="s">
+        <v>39</v>
+      </c>
+      <c r="F6" t="s">
+        <v>40</v>
+      </c>
+      <c r="G6" t="s">
+        <v>41</v>
+      </c>
+      <c r="H6" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="7" spans="1:8" x14ac:dyDescent="0.4">
+      <c r="A7" t="s">
+        <v>8</v>
+      </c>
+      <c r="B7" t="s">
         <v>24</v>
       </c>
-    </row>
-    <row r="7" spans="1:8">
-      <c r="A7" t="s">
-        <v>8</v>
-      </c>
-      <c r="B7" t="s">
+      <c r="C7" t="s">
         <v>25</v>
       </c>
-      <c r="C7" t="s">
+      <c r="D7" t="s">
         <v>26</v>
       </c>
-      <c r="D7" t="s">
+      <c r="E7" t="s">
+        <v>39</v>
+      </c>
+      <c r="F7" t="s">
+        <v>40</v>
+      </c>
+      <c r="G7" t="s">
+        <v>41</v>
+      </c>
+      <c r="H7" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="8" spans="1:8" x14ac:dyDescent="0.4">
+      <c r="A8" t="s">
+        <v>8</v>
+      </c>
+      <c r="B8" t="s">
         <v>27</v>
       </c>
-    </row>
-    <row r="8" spans="1:8">
-      <c r="A8" t="s">
-        <v>8</v>
-      </c>
-      <c r="B8" t="s">
+      <c r="C8" t="s">
         <v>28</v>
       </c>
-      <c r="C8" t="s">
+      <c r="D8" t="s">
         <v>29</v>
       </c>
-      <c r="D8" t="s">
+      <c r="E8" t="s">
+        <v>39</v>
+      </c>
+      <c r="F8" t="s">
+        <v>40</v>
+      </c>
+      <c r="G8" t="s">
+        <v>41</v>
+      </c>
+      <c r="H8" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="9" spans="1:8" x14ac:dyDescent="0.4">
+      <c r="A9" t="s">
+        <v>8</v>
+      </c>
+      <c r="B9" t="s">
         <v>30</v>
       </c>
-    </row>
-    <row r="9" spans="1:8">
-      <c r="A9" t="s">
-        <v>8</v>
-      </c>
-      <c r="B9" t="s">
+      <c r="C9" t="s">
         <v>31</v>
       </c>
-      <c r="C9" t="s">
+      <c r="D9" t="s">
         <v>32</v>
       </c>
-      <c r="D9" t="s">
+      <c r="E9" t="s">
+        <v>72</v>
+      </c>
+      <c r="F9" t="s">
+        <v>40</v>
+      </c>
+      <c r="G9" t="s">
+        <v>41</v>
+      </c>
+      <c r="H9" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="10" spans="1:8" x14ac:dyDescent="0.4">
+      <c r="A10" t="s">
+        <v>8</v>
+      </c>
+      <c r="B10" t="s">
         <v>33</v>
       </c>
-    </row>
-    <row r="10" spans="1:8">
-      <c r="A10" t="s">
-        <v>8</v>
-      </c>
-      <c r="B10" t="s">
+      <c r="C10" t="s">
         <v>34</v>
       </c>
-      <c r="C10" t="s">
+      <c r="D10" t="s">
         <v>35</v>
       </c>
-      <c r="D10" t="s">
+      <c r="E10" t="s">
+        <v>39</v>
+      </c>
+      <c r="F10" t="s">
+        <v>40</v>
+      </c>
+      <c r="G10" t="s">
+        <v>41</v>
+      </c>
+      <c r="H10" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="11" spans="1:8" x14ac:dyDescent="0.4">
+      <c r="A11" t="s">
+        <v>8</v>
+      </c>
+      <c r="B11" t="s">
         <v>36</v>
       </c>
-    </row>
-    <row r="11" spans="1:8">
-      <c r="A11" t="s">
-        <v>8</v>
-      </c>
-      <c r="B11" t="s">
+      <c r="C11" t="s">
         <v>37</v>
       </c>
-      <c r="C11" t="s">
+      <c r="D11" t="s">
         <v>38</v>
       </c>
-      <c r="D11" t="s">
-        <v>39</v>
-      </c>
       <c r="E11" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="F11" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="G11" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="H11" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="12" spans="1:8" x14ac:dyDescent="0.4">
+      <c r="A12" t="s">
+        <v>8</v>
+      </c>
+      <c r="B12" t="s">
         <v>43</v>
       </c>
-    </row>
-    <row r="12" spans="1:8">
-      <c r="A12" t="s">
-        <v>8</v>
-      </c>
-      <c r="B12" t="s">
+      <c r="C12" t="s">
         <v>44</v>
       </c>
-      <c r="C12" t="s">
+      <c r="D12" t="s">
         <v>45</v>
       </c>
-      <c r="D12" t="s">
+      <c r="E12" t="s">
+        <v>39</v>
+      </c>
+      <c r="F12" t="s">
+        <v>40</v>
+      </c>
+      <c r="G12" t="s">
+        <v>41</v>
+      </c>
+      <c r="H12" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="13" spans="1:8" x14ac:dyDescent="0.4">
+      <c r="A13" t="s">
+        <v>8</v>
+      </c>
+      <c r="B13" t="s">
         <v>46</v>
       </c>
-      <c r="E12" t="s">
-        <v>40</v>
-      </c>
-      <c r="F12" t="s">
-        <v>41</v>
-      </c>
-      <c r="G12" t="s">
-        <v>42</v>
-      </c>
-      <c r="H12" t="s">
-        <v>43</v>
-      </c>
-    </row>
-    <row r="13" spans="1:8">
-      <c r="A13" t="s">
-        <v>8</v>
-      </c>
-      <c r="B13" t="s">
+      <c r="C13" t="s">
         <v>47</v>
       </c>
-      <c r="C13" t="s">
+      <c r="D13" t="s">
         <v>48</v>
       </c>
-      <c r="D13" t="s">
+      <c r="E13" t="s">
+        <v>39</v>
+      </c>
+      <c r="F13" t="s">
+        <v>40</v>
+      </c>
+      <c r="G13" t="s">
+        <v>41</v>
+      </c>
+      <c r="H13" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="14" spans="1:8" x14ac:dyDescent="0.4">
+      <c r="A14" t="s">
+        <v>8</v>
+      </c>
+      <c r="B14" t="s">
         <v>49</v>
       </c>
-      <c r="E13" t="s">
-        <v>40</v>
-      </c>
-      <c r="F13" t="s">
-        <v>41</v>
-      </c>
-      <c r="G13" t="s">
-        <v>42</v>
-      </c>
-      <c r="H13" t="s">
-        <v>43</v>
-      </c>
-    </row>
-    <row r="14" spans="1:8">
-      <c r="A14" t="s">
-        <v>8</v>
-      </c>
-      <c r="B14" t="s">
+      <c r="C14" t="s">
         <v>50</v>
       </c>
-      <c r="C14" t="s">
+      <c r="D14" t="s">
         <v>51</v>
       </c>
-      <c r="D14" t="s">
+      <c r="E14" t="s">
+        <v>39</v>
+      </c>
+      <c r="F14" t="s">
+        <v>40</v>
+      </c>
+      <c r="G14" t="s">
+        <v>41</v>
+      </c>
+      <c r="H14" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="15" spans="1:8" x14ac:dyDescent="0.4">
+      <c r="A15" t="s">
+        <v>8</v>
+      </c>
+      <c r="B15" t="s">
         <v>52</v>
       </c>
-      <c r="E14" t="s">
-        <v>40</v>
-      </c>
-      <c r="F14" t="s">
-        <v>41</v>
-      </c>
-      <c r="G14" t="s">
-        <v>42</v>
-      </c>
-      <c r="H14" t="s">
-        <v>43</v>
-      </c>
-    </row>
-    <row r="15" spans="1:8">
-      <c r="A15" t="s">
-        <v>8</v>
-      </c>
-      <c r="B15" t="s">
+      <c r="C15" t="s">
         <v>53</v>
       </c>
-      <c r="C15" t="s">
+      <c r="D15" t="s">
         <v>54</v>
       </c>
-      <c r="D15" t="s">
+      <c r="E15" t="s">
+        <v>39</v>
+      </c>
+      <c r="F15" t="s">
+        <v>40</v>
+      </c>
+      <c r="G15" t="s">
+        <v>41</v>
+      </c>
+      <c r="H15" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="16" spans="1:8" x14ac:dyDescent="0.4">
+      <c r="A16" t="s">
+        <v>8</v>
+      </c>
+      <c r="B16" t="s">
         <v>55</v>
       </c>
-      <c r="E15" t="s">
-        <v>40</v>
-      </c>
-      <c r="F15" t="s">
-        <v>41</v>
-      </c>
-      <c r="G15" t="s">
-        <v>42</v>
-      </c>
-      <c r="H15" t="s">
-        <v>43</v>
-      </c>
-    </row>
-    <row r="16" spans="1:8">
-      <c r="A16" t="s">
-        <v>8</v>
-      </c>
-      <c r="B16" t="s">
+      <c r="C16" t="s">
         <v>56</v>
       </c>
-      <c r="C16" t="s">
+      <c r="D16" t="s">
         <v>57</v>
       </c>
-      <c r="D16" t="s">
+      <c r="E16" t="s">
+        <v>39</v>
+      </c>
+      <c r="F16" t="s">
+        <v>40</v>
+      </c>
+      <c r="G16" t="s">
+        <v>41</v>
+      </c>
+      <c r="H16" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="17" spans="1:8" x14ac:dyDescent="0.4">
+      <c r="A17" t="s">
+        <v>8</v>
+      </c>
+      <c r="B17" t="s">
+        <v>67</v>
+      </c>
+      <c r="D17" t="s">
+        <v>73</v>
+      </c>
+      <c r="E17" t="s">
+        <v>39</v>
+      </c>
+      <c r="F17" t="s">
+        <v>40</v>
+      </c>
+      <c r="G17" t="s">
+        <v>41</v>
+      </c>
+      <c r="H17" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="18" spans="1:8" x14ac:dyDescent="0.4">
+      <c r="A18" t="s">
+        <v>8</v>
+      </c>
+      <c r="B18" t="s">
         <v>58</v>
       </c>
-      <c r="E16" t="s">
-        <v>40</v>
-      </c>
-      <c r="F16" t="s">
-        <v>41</v>
-      </c>
-      <c r="G16" t="s">
-        <v>42</v>
-      </c>
-      <c r="H16" t="s">
-        <v>43</v>
-      </c>
-    </row>
-    <row r="17" spans="1:8">
-      <c r="A17" t="s">
-        <v>8</v>
-      </c>
-      <c r="B17" t="s">
+      <c r="C18" t="s">
         <v>59</v>
       </c>
-      <c r="C17" t="s">
+      <c r="D18" t="s">
         <v>60</v>
       </c>
-      <c r="D17" t="s">
+      <c r="E18" t="s">
+        <v>39</v>
+      </c>
+      <c r="F18" t="s">
+        <v>40</v>
+      </c>
+      <c r="G18" t="s">
+        <v>41</v>
+      </c>
+      <c r="H18" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="19" spans="1:8" x14ac:dyDescent="0.4">
+      <c r="A19" t="s">
+        <v>8</v>
+      </c>
+      <c r="B19" t="s">
         <v>61</v>
       </c>
-      <c r="E17" t="s">
-        <v>40</v>
-      </c>
-      <c r="F17" t="s">
-        <v>41</v>
-      </c>
-      <c r="G17" t="s">
-        <v>42</v>
-      </c>
-      <c r="H17" t="s">
-        <v>43</v>
-      </c>
-    </row>
-    <row r="18" spans="1:8">
-      <c r="A18" t="s">
-        <v>8</v>
-      </c>
-      <c r="B18" t="s">
+      <c r="C19" t="s">
         <v>62</v>
       </c>
-      <c r="C18" t="s">
+      <c r="D19" t="s">
         <v>63</v>
       </c>
-      <c r="D18" t="s">
+      <c r="E19" t="s">
+        <v>39</v>
+      </c>
+      <c r="F19" t="s">
+        <v>40</v>
+      </c>
+      <c r="G19" t="s">
+        <v>41</v>
+      </c>
+      <c r="H19" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="20" spans="1:8" x14ac:dyDescent="0.4">
+      <c r="A20" t="s">
+        <v>8</v>
+      </c>
+      <c r="B20" t="s">
         <v>64</v>
       </c>
-      <c r="E18" t="s">
-        <v>40</v>
-      </c>
-      <c r="F18" t="s">
-        <v>41</v>
-      </c>
-      <c r="G18" t="s">
-        <v>42</v>
-      </c>
-      <c r="H18" t="s">
-        <v>43</v>
-      </c>
-    </row>
-    <row r="19" spans="1:8">
-      <c r="A19" t="s">
-        <v>8</v>
-      </c>
-      <c r="B19" t="s">
+      <c r="C20" t="s">
         <v>65</v>
       </c>
-      <c r="C19" t="s">
+      <c r="D20" t="s">
         <v>66</v>
       </c>
-      <c r="D19" t="s">
-        <v>67</v>
-      </c>
-      <c r="E19" t="s">
-        <v>40</v>
-      </c>
-      <c r="F19" t="s">
-        <v>41</v>
-      </c>
-      <c r="G19" t="s">
-        <v>42</v>
-      </c>
-      <c r="H19" t="s">
-        <v>43</v>
+      <c r="E20" t="s">
+        <v>39</v>
+      </c>
+      <c r="F20" t="s">
+        <v>40</v>
+      </c>
+      <c r="G20" t="s">
+        <v>41</v>
+      </c>
+      <c r="H20" t="s">
+        <v>42</v>
       </c>
     </row>
   </sheetData>
+  <phoneticPr fontId="1" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>